<commit_message>
Suskaičiuota Aerodinamika iki izokinetiškumo
</commit_message>
<xml_diff>
--- a/Ivestis2.xlsx
+++ b/Ivestis2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agentura2020.sharepoint.com/sites/VidurioLietuvosaplinkostyrimuskyrius/Bendrai naudojami dokumentai/EB7-014 Darbuotojų failai/Tomo/Python 3.14.3/Skaiciavimai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{A643DED9-AFCA-45B4-88D7-0278F4B57F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FBEC764-D3B5-4E6C-B35A-438B078D31B3}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="13_ncr:1_{A643DED9-AFCA-45B4-88D7-0278F4B57F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6025435-91FC-459E-B688-2967D1DEEE39}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="3" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="4" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -2681,6 +2681,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -2761,31 +2786,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2796,6 +2796,42 @@
     <xf numFmtId="169" fontId="4" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2811,42 +2847,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -3253,6 +3253,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B3F6816-A3F5-4347-BE94-F213DC59E543}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A3:AB31"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3282,31 +3285,31 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="D3" s="258" t="s">
+      <c r="D3" s="265" t="s">
         <v>111</v>
       </c>
-      <c r="E3" s="258"/>
-      <c r="F3" s="258"/>
-      <c r="G3" s="258"/>
-      <c r="H3" s="258"/>
-      <c r="I3" s="258"/>
-      <c r="J3" s="258"/>
-      <c r="K3" s="258"/>
-      <c r="L3" s="258"/>
-      <c r="M3" s="258"/>
-      <c r="N3" s="258"/>
-      <c r="O3" s="258"/>
-      <c r="P3" s="258"/>
-      <c r="Q3" s="258"/>
-      <c r="R3" s="258"/>
-      <c r="S3" s="258"/>
-      <c r="T3" s="258"/>
-      <c r="U3" s="258"/>
-      <c r="V3" s="258"/>
-      <c r="W3" s="258"/>
-      <c r="X3" s="258"/>
-      <c r="Y3" s="258"/>
-      <c r="Z3" s="258"/>
+      <c r="E3" s="265"/>
+      <c r="F3" s="265"/>
+      <c r="G3" s="265"/>
+      <c r="H3" s="265"/>
+      <c r="I3" s="265"/>
+      <c r="J3" s="265"/>
+      <c r="K3" s="265"/>
+      <c r="L3" s="265"/>
+      <c r="M3" s="265"/>
+      <c r="N3" s="265"/>
+      <c r="O3" s="265"/>
+      <c r="P3" s="265"/>
+      <c r="Q3" s="265"/>
+      <c r="R3" s="265"/>
+      <c r="S3" s="265"/>
+      <c r="T3" s="265"/>
+      <c r="U3" s="265"/>
+      <c r="V3" s="265"/>
+      <c r="W3" s="265"/>
+      <c r="X3" s="265"/>
+      <c r="Y3" s="265"/>
+      <c r="Z3" s="265"/>
     </row>
     <row r="5" spans="1:28" s="10" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
@@ -3395,13 +3398,13 @@
       </c>
     </row>
     <row r="6" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="259">
+      <c r="A6" s="266">
         <v>46210</v>
       </c>
-      <c r="B6" s="260">
+      <c r="B6" s="267">
         <v>7</v>
       </c>
-      <c r="C6" s="261" t="s">
+      <c r="C6" s="268" t="s">
         <v>140</v>
       </c>
       <c r="D6" s="151">
@@ -3492,14 +3495,14 @@
         <f>Aerodinamika!G31</f>
         <v>1.2973599999999996</v>
       </c>
-      <c r="AB6" s="256" t="s">
+      <c r="AB6" s="263" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="260"/>
-      <c r="B7" s="260"/>
-      <c r="C7" s="261"/>
+      <c r="A7" s="267"/>
+      <c r="B7" s="267"/>
+      <c r="C7" s="268"/>
       <c r="D7" s="151">
         <v>2</v>
       </c>
@@ -3584,12 +3587,12 @@
         <f>O6*X7</f>
         <v>0.33485669081573011</v>
       </c>
-      <c r="AB7" s="257"/>
+      <c r="AB7" s="264"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="260"/>
-      <c r="B8" s="260"/>
-      <c r="C8" s="261"/>
+      <c r="A8" s="267"/>
+      <c r="B8" s="267"/>
+      <c r="C8" s="268"/>
       <c r="D8" s="173">
         <v>3</v>
       </c>
@@ -3640,9 +3643,9 @@
       <c r="S8" s="180"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A9" s="260"/>
-      <c r="B9" s="260"/>
-      <c r="C9" s="261"/>
+      <c r="A9" s="267"/>
+      <c r="B9" s="267"/>
+      <c r="C9" s="268"/>
       <c r="D9" s="151">
         <v>4</v>
       </c>
@@ -3697,9 +3700,9 @@
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A10" s="260"/>
-      <c r="B10" s="260"/>
-      <c r="C10" s="261"/>
+      <c r="A10" s="267"/>
+      <c r="B10" s="267"/>
+      <c r="C10" s="268"/>
       <c r="D10" s="151">
         <v>5</v>
       </c>
@@ -3743,9 +3746,9 @@
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="260"/>
-      <c r="B11" s="260"/>
-      <c r="C11" s="261"/>
+      <c r="A11" s="267"/>
+      <c r="B11" s="267"/>
+      <c r="C11" s="268"/>
       <c r="D11" s="151">
         <v>6</v>
       </c>
@@ -3789,9 +3792,9 @@
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A12" s="260"/>
-      <c r="B12" s="260"/>
-      <c r="C12" s="261"/>
+      <c r="A12" s="267"/>
+      <c r="B12" s="267"/>
+      <c r="C12" s="268"/>
       <c r="D12" s="151">
         <v>7</v>
       </c>
@@ -3835,9 +3838,9 @@
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="260"/>
-      <c r="B13" s="260"/>
-      <c r="C13" s="261"/>
+      <c r="A13" s="267"/>
+      <c r="B13" s="267"/>
+      <c r="C13" s="268"/>
       <c r="D13" s="151">
         <v>8</v>
       </c>
@@ -3882,9 +3885,9 @@
       <c r="O13" s="145"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="260"/>
-      <c r="B14" s="260"/>
-      <c r="C14" s="261"/>
+      <c r="A14" s="267"/>
+      <c r="B14" s="267"/>
+      <c r="C14" s="268"/>
       <c r="D14" s="151">
         <v>9</v>
       </c>
@@ -3960,18 +3963,18 @@
       <c r="D16" s="173" t="s">
         <v>136</v>
       </c>
-      <c r="E16" s="262" t="s">
+      <c r="E16" s="269" t="s">
         <v>137</v>
       </c>
-      <c r="F16" s="263"/>
-      <c r="G16" s="263"/>
-      <c r="H16" s="263"/>
-      <c r="I16" s="263"/>
-      <c r="J16" s="263"/>
-      <c r="K16" s="263"/>
-      <c r="L16" s="263"/>
-      <c r="M16" s="263"/>
-      <c r="N16" s="264"/>
+      <c r="F16" s="270"/>
+      <c r="G16" s="270"/>
+      <c r="H16" s="270"/>
+      <c r="I16" s="270"/>
+      <c r="J16" s="270"/>
+      <c r="K16" s="270"/>
+      <c r="L16" s="270"/>
+      <c r="M16" s="270"/>
+      <c r="N16" s="271"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="150"/>
@@ -4006,31 +4009,31 @@
       <c r="A20" s="184"/>
       <c r="B20" s="184"/>
       <c r="C20" s="184"/>
-      <c r="D20" s="265" t="s">
+      <c r="D20" s="272" t="s">
         <v>139</v>
       </c>
-      <c r="E20" s="258"/>
-      <c r="F20" s="258"/>
-      <c r="G20" s="258"/>
-      <c r="H20" s="258"/>
-      <c r="I20" s="258"/>
-      <c r="J20" s="258"/>
-      <c r="K20" s="258"/>
-      <c r="L20" s="258"/>
-      <c r="M20" s="258"/>
-      <c r="N20" s="258"/>
-      <c r="O20" s="258"/>
-      <c r="P20" s="258"/>
-      <c r="Q20" s="258"/>
-      <c r="R20" s="258"/>
-      <c r="S20" s="258"/>
-      <c r="T20" s="258"/>
-      <c r="U20" s="258"/>
-      <c r="V20" s="258"/>
-      <c r="W20" s="258"/>
-      <c r="X20" s="258"/>
-      <c r="Y20" s="258"/>
-      <c r="Z20" s="258"/>
+      <c r="E20" s="265"/>
+      <c r="F20" s="265"/>
+      <c r="G20" s="265"/>
+      <c r="H20" s="265"/>
+      <c r="I20" s="265"/>
+      <c r="J20" s="265"/>
+      <c r="K20" s="265"/>
+      <c r="L20" s="265"/>
+      <c r="M20" s="265"/>
+      <c r="N20" s="265"/>
+      <c r="O20" s="265"/>
+      <c r="P20" s="265"/>
+      <c r="Q20" s="265"/>
+      <c r="R20" s="265"/>
+      <c r="S20" s="265"/>
+      <c r="T20" s="265"/>
+      <c r="U20" s="265"/>
+      <c r="V20" s="265"/>
+      <c r="W20" s="265"/>
+      <c r="X20" s="265"/>
+      <c r="Y20" s="265"/>
+      <c r="Z20" s="265"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" s="150"/>
@@ -4136,9 +4139,9 @@
       </c>
     </row>
     <row r="23" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="266"/>
-      <c r="B23" s="266"/>
-      <c r="C23" s="266"/>
+      <c r="A23" s="273"/>
+      <c r="B23" s="273"/>
+      <c r="C23" s="273"/>
       <c r="D23" s="151">
         <v>3</v>
       </c>
@@ -4215,12 +4218,12 @@
       <c r="AA23" s="165">
         <v>1.35</v>
       </c>
-      <c r="AB23" s="256"/>
+      <c r="AB23" s="263"/>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A24" s="267"/>
-      <c r="B24" s="267"/>
-      <c r="C24" s="267"/>
+      <c r="A24" s="274"/>
+      <c r="B24" s="274"/>
+      <c r="C24" s="274"/>
       <c r="D24" s="151">
         <v>15</v>
       </c>
@@ -4291,12 +4294,12 @@
         <f>O23*X24</f>
         <v>1.0498709847610572</v>
       </c>
-      <c r="AB24" s="257"/>
+      <c r="AB24" s="264"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A25" s="267"/>
-      <c r="B25" s="267"/>
-      <c r="C25" s="267"/>
+      <c r="A25" s="274"/>
+      <c r="B25" s="274"/>
+      <c r="C25" s="274"/>
       <c r="D25" s="173">
         <v>27</v>
       </c>
@@ -4335,9 +4338,9 @@
       <c r="S25" s="180"/>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A26" s="267"/>
-      <c r="B26" s="267"/>
-      <c r="C26" s="267"/>
+      <c r="A26" s="274"/>
+      <c r="B26" s="274"/>
+      <c r="C26" s="274"/>
       <c r="D26" s="151">
         <v>4</v>
       </c>
@@ -4380,9 +4383,9 @@
       </c>
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A27" s="267"/>
-      <c r="B27" s="267"/>
-      <c r="C27" s="267"/>
+      <c r="A27" s="274"/>
+      <c r="B27" s="274"/>
+      <c r="C27" s="274"/>
       <c r="D27" s="151">
         <v>5</v>
       </c>
@@ -4414,9 +4417,9 @@
       </c>
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A28" s="267"/>
-      <c r="B28" s="267"/>
-      <c r="C28" s="267"/>
+      <c r="A28" s="274"/>
+      <c r="B28" s="274"/>
+      <c r="C28" s="274"/>
       <c r="D28" s="151">
         <v>6</v>
       </c>
@@ -4448,9 +4451,9 @@
       </c>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A29" s="267"/>
-      <c r="B29" s="267"/>
-      <c r="C29" s="267"/>
+      <c r="A29" s="274"/>
+      <c r="B29" s="274"/>
+      <c r="C29" s="274"/>
       <c r="D29" s="151">
         <v>7</v>
       </c>
@@ -4482,9 +4485,9 @@
       </c>
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A30" s="267"/>
-      <c r="B30" s="267"/>
-      <c r="C30" s="267"/>
+      <c r="A30" s="274"/>
+      <c r="B30" s="274"/>
+      <c r="C30" s="274"/>
       <c r="D30" s="151">
         <v>8</v>
       </c>
@@ -4517,9 +4520,9 @@
       <c r="O30" s="145"/>
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A31" s="268"/>
-      <c r="B31" s="268"/>
-      <c r="C31" s="268"/>
+      <c r="A31" s="275"/>
+      <c r="B31" s="275"/>
+      <c r="C31" s="275"/>
       <c r="D31" s="151">
         <v>9</v>
       </c>
@@ -4570,6 +4573,7 @@
     <mergeCell ref="C23:C31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="30" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4613,18 +4617,18 @@
       <c r="I2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="269" t="s">
+      <c r="A3" s="276" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="269"/>
-      <c r="C3" s="269"/>
-      <c r="D3" s="269"/>
-      <c r="E3" s="269"/>
-      <c r="F3" s="269"/>
-      <c r="G3" s="269"/>
-      <c r="H3" s="269"/>
-      <c r="I3" s="269"/>
-      <c r="J3" s="269"/>
+      <c r="B3" s="276"/>
+      <c r="C3" s="276"/>
+      <c r="D3" s="276"/>
+      <c r="E3" s="276"/>
+      <c r="F3" s="276"/>
+      <c r="G3" s="276"/>
+      <c r="H3" s="276"/>
+      <c r="I3" s="276"/>
+      <c r="J3" s="276"/>
     </row>
     <row r="4" spans="1:12" ht="14" x14ac:dyDescent="0.3">
       <c r="A4" s="10"/>
@@ -4771,46 +4775,46 @@
       <c r="L10" s="47"/>
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H11" s="270" t="s">
+      <c r="H11" s="277" t="s">
         <v>31</v>
       </c>
-      <c r="I11" s="273" t="s">
+      <c r="I11" s="280" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H12" s="271"/>
-      <c r="I12" s="274"/>
+      <c r="H12" s="278"/>
+      <c r="I12" s="281"/>
     </row>
     <row r="13" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H13" s="271"/>
-      <c r="I13" s="274"/>
+      <c r="H13" s="278"/>
+      <c r="I13" s="281"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H14" s="271"/>
-      <c r="I14" s="274"/>
+      <c r="H14" s="278"/>
+      <c r="I14" s="281"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H15" s="271"/>
-      <c r="I15" s="274"/>
+      <c r="H15" s="278"/>
+      <c r="I15" s="281"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H16" s="271"/>
-      <c r="I16" s="274"/>
+      <c r="H16" s="278"/>
+      <c r="I16" s="281"/>
     </row>
     <row r="17" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H17" s="271"/>
-      <c r="I17" s="274"/>
+      <c r="H17" s="278"/>
+      <c r="I17" s="281"/>
     </row>
     <row r="18" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H18" s="272"/>
-      <c r="I18" s="274"/>
+      <c r="H18" s="279"/>
+      <c r="I18" s="281"/>
     </row>
     <row r="19" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I19" s="274"/>
+      <c r="I19" s="281"/>
     </row>
     <row r="20" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I20" s="275"/>
+      <c r="I20" s="282"/>
     </row>
     <row r="21" spans="8:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I21" s="59"/>
@@ -4836,6 +4840,7 @@
     <mergeCell ref="I11:I20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4875,35 +4880,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="281" t="s">
+      <c r="C1" s="261" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="281"/>
+      <c r="D1" s="261"/>
       <c r="E1" s="15"/>
       <c r="S1" s="16"/>
     </row>
     <row r="2" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="282" t="s">
+      <c r="A2" s="262" t="s">
         <v>101</v>
       </c>
-      <c r="B2" s="282"/>
-      <c r="C2" s="282"/>
-      <c r="D2" s="282"/>
-      <c r="E2" s="282"/>
-      <c r="F2" s="282"/>
-      <c r="G2" s="282"/>
-      <c r="H2" s="282"/>
-      <c r="I2" s="282"/>
-      <c r="J2" s="282"/>
-      <c r="K2" s="282"/>
-      <c r="L2" s="282"/>
-      <c r="M2" s="282"/>
-      <c r="N2" s="282"/>
-      <c r="O2" s="282"/>
-      <c r="P2" s="282"/>
-      <c r="Q2" s="282"/>
-      <c r="R2" s="282"/>
-      <c r="S2" s="282"/>
+      <c r="B2" s="262"/>
+      <c r="C2" s="262"/>
+      <c r="D2" s="262"/>
+      <c r="E2" s="262"/>
+      <c r="F2" s="262"/>
+      <c r="G2" s="262"/>
+      <c r="H2" s="262"/>
+      <c r="I2" s="262"/>
+      <c r="J2" s="262"/>
+      <c r="K2" s="262"/>
+      <c r="L2" s="262"/>
+      <c r="M2" s="262"/>
+      <c r="N2" s="262"/>
+      <c r="O2" s="262"/>
+      <c r="P2" s="262"/>
+      <c r="Q2" s="262"/>
+      <c r="R2" s="262"/>
+      <c r="S2" s="262"/>
     </row>
     <row r="3" spans="1:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
@@ -5011,7 +5016,7 @@
       <c r="B6" s="52">
         <v>1</v>
       </c>
-      <c r="C6" s="277" t="str">
+      <c r="C6" s="257" t="str">
         <f>Greitis!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5091,7 +5096,7 @@
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" s="37"/>
       <c r="B7" s="34"/>
-      <c r="C7" s="278"/>
+      <c r="C7" s="258"/>
       <c r="D7" s="19"/>
       <c r="E7" s="20"/>
       <c r="F7" s="216">
@@ -5162,7 +5167,7 @@
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" s="37"/>
       <c r="B8" s="34"/>
-      <c r="C8" s="278"/>
+      <c r="C8" s="258"/>
       <c r="D8" s="19"/>
       <c r="E8" s="20"/>
       <c r="F8" s="216">
@@ -5233,7 +5238,7 @@
     <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" s="51"/>
       <c r="B9" s="51"/>
-      <c r="C9" s="278"/>
+      <c r="C9" s="258"/>
       <c r="D9" s="51"/>
       <c r="E9" s="51"/>
       <c r="F9" s="216">
@@ -5307,7 +5312,7 @@
     <row r="10" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="51"/>
       <c r="B10" s="51"/>
-      <c r="C10" s="278"/>
+      <c r="C10" s="258"/>
       <c r="D10" s="51"/>
       <c r="E10" s="51"/>
       <c r="F10" s="216">
@@ -5357,13 +5362,13 @@
       </c>
       <c r="R10" s="51"/>
       <c r="S10" s="51"/>
-      <c r="T10" s="280" t="s">
+      <c r="T10" s="260" t="s">
         <v>33</v>
       </c>
-      <c r="U10" s="280" t="s">
+      <c r="U10" s="260" t="s">
         <v>34</v>
       </c>
-      <c r="V10" s="276" t="s">
+      <c r="V10" s="256" t="s">
         <v>41</v>
       </c>
       <c r="X10" s="211">
@@ -5378,7 +5383,7 @@
     <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" s="51"/>
       <c r="B11" s="51"/>
-      <c r="C11" s="278"/>
+      <c r="C11" s="258"/>
       <c r="D11" s="51"/>
       <c r="E11" s="51"/>
       <c r="F11" s="216">
@@ -5428,9 +5433,9 @@
       </c>
       <c r="R11" s="51"/>
       <c r="S11" s="51"/>
-      <c r="T11" s="280"/>
-      <c r="U11" s="280"/>
-      <c r="V11" s="276"/>
+      <c r="T11" s="260"/>
+      <c r="U11" s="260"/>
+      <c r="V11" s="256"/>
       <c r="X11" s="211">
         <f>Greitis!E11</f>
         <v>0.12</v>
@@ -5443,7 +5448,7 @@
     <row r="12" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="51"/>
       <c r="B12" s="51"/>
-      <c r="C12" s="278"/>
+      <c r="C12" s="258"/>
       <c r="D12" s="51"/>
       <c r="E12" s="51"/>
       <c r="F12" s="216">
@@ -5493,9 +5498,9 @@
       </c>
       <c r="R12" s="51"/>
       <c r="S12" s="51"/>
-      <c r="T12" s="280"/>
-      <c r="U12" s="280"/>
-      <c r="V12" s="276"/>
+      <c r="T12" s="260"/>
+      <c r="U12" s="260"/>
+      <c r="V12" s="256"/>
       <c r="X12" s="211">
         <f>Greitis!E12</f>
         <v>0.12</v>
@@ -5508,7 +5513,7 @@
     <row r="13" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="51"/>
       <c r="B13" s="51"/>
-      <c r="C13" s="278"/>
+      <c r="C13" s="258"/>
       <c r="D13" s="51"/>
       <c r="E13" s="51"/>
       <c r="F13" s="216">
@@ -5570,7 +5575,7 @@
     <row r="14" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="36"/>
       <c r="B14" s="36"/>
-      <c r="C14" s="279"/>
+      <c r="C14" s="259"/>
       <c r="D14" s="36"/>
       <c r="E14" s="36"/>
       <c r="F14" s="216">
@@ -5668,7 +5673,7 @@
         <f t="shared" si="27"/>
         <v>1</v>
       </c>
-      <c r="C19" s="277" t="str">
+      <c r="C19" s="257" t="str">
         <f t="shared" si="27"/>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -5744,7 +5749,7 @@
     <row r="20" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A20" s="37"/>
       <c r="B20" s="34"/>
-      <c r="C20" s="278"/>
+      <c r="C20" s="258"/>
       <c r="D20" s="19"/>
       <c r="E20" s="20"/>
       <c r="F20" s="216">
@@ -5806,7 +5811,7 @@
     <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21" s="37"/>
       <c r="B21" s="34"/>
-      <c r="C21" s="278"/>
+      <c r="C21" s="258"/>
       <c r="D21" s="19"/>
       <c r="E21" s="20"/>
       <c r="F21" s="216">
@@ -5868,7 +5873,7 @@
     <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22" s="51"/>
       <c r="B22" s="51"/>
-      <c r="C22" s="278"/>
+      <c r="C22" s="258"/>
       <c r="D22" s="51"/>
       <c r="E22" s="51"/>
       <c r="F22" s="216">
@@ -5930,7 +5935,7 @@
     <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23" s="51"/>
       <c r="B23" s="51"/>
-      <c r="C23" s="278"/>
+      <c r="C23" s="258"/>
       <c r="D23" s="51"/>
       <c r="E23" s="51"/>
       <c r="F23" s="216">
@@ -5992,7 +5997,7 @@
     <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" s="51"/>
       <c r="B24" s="51"/>
-      <c r="C24" s="278"/>
+      <c r="C24" s="258"/>
       <c r="D24" s="51"/>
       <c r="E24" s="51"/>
       <c r="F24" s="216">
@@ -6054,7 +6059,7 @@
     <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" s="51"/>
       <c r="B25" s="51"/>
-      <c r="C25" s="278"/>
+      <c r="C25" s="258"/>
       <c r="D25" s="51"/>
       <c r="E25" s="51"/>
       <c r="F25" s="216">
@@ -6116,7 +6121,7 @@
     <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" s="51"/>
       <c r="B26" s="51"/>
-      <c r="C26" s="278"/>
+      <c r="C26" s="258"/>
       <c r="D26" s="51"/>
       <c r="E26" s="51"/>
       <c r="F26" s="216">
@@ -6178,7 +6183,7 @@
     <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27" s="36"/>
       <c r="B27" s="36"/>
-      <c r="C27" s="279"/>
+      <c r="C27" s="259"/>
       <c r="D27" s="36"/>
       <c r="E27" s="36"/>
       <c r="F27" s="216">
@@ -6315,7 +6320,7 @@
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.19685039370078741" right="0" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="66" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="63" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;CPuslapių &amp;P &amp;R&amp;"Times New Roman,Paryškintasis"E5-5_02         
 2022-02-01, EV</oddFooter>
@@ -6349,10 +6354,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="281" t="s">
+      <c r="C1" s="261" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="281"/>
+      <c r="D1" s="261"/>
       <c r="Q1" s="16"/>
     </row>
     <row r="2" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -6430,7 +6435,7 @@
         <f>Paėmimas!B6</f>
         <v>1</v>
       </c>
-      <c r="C6" s="277" t="str">
+      <c r="C6" s="257" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6482,7 +6487,7 @@
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="61"/>
       <c r="B7" s="23"/>
-      <c r="C7" s="278"/>
+      <c r="C7" s="258"/>
       <c r="D7" s="224">
         <f>Paėmimas!L7</f>
         <v>0.05</v>
@@ -6519,7 +6524,7 @@
     <row r="8" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="61"/>
       <c r="B8" s="23"/>
-      <c r="C8" s="278"/>
+      <c r="C8" s="258"/>
       <c r="D8" s="224">
         <f>Paėmimas!L8</f>
         <v>0.05</v>
@@ -6556,7 +6561,7 @@
     <row r="9" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="61"/>
       <c r="B9" s="23"/>
-      <c r="C9" s="278"/>
+      <c r="C9" s="258"/>
       <c r="D9" s="224">
         <f>Paėmimas!L9</f>
         <v>0.05</v>
@@ -6593,7 +6598,7 @@
     <row r="10" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="61"/>
       <c r="B10" s="23"/>
-      <c r="C10" s="278"/>
+      <c r="C10" s="258"/>
       <c r="D10" s="224">
         <f>Paėmimas!L10</f>
         <v>0.05</v>
@@ -6630,7 +6635,7 @@
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="61"/>
       <c r="B11" s="23"/>
-      <c r="C11" s="278"/>
+      <c r="C11" s="258"/>
       <c r="D11" s="224">
         <f>Paėmimas!L11</f>
         <v>0.05</v>
@@ -6667,7 +6672,7 @@
     <row r="12" spans="1:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="61"/>
       <c r="B12" s="23"/>
-      <c r="C12" s="278"/>
+      <c r="C12" s="258"/>
       <c r="D12" s="224">
         <f>Paėmimas!L12</f>
         <v>0.05</v>
@@ -6704,7 +6709,7 @@
     <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="61"/>
       <c r="B13" s="23"/>
-      <c r="C13" s="278"/>
+      <c r="C13" s="258"/>
       <c r="D13" s="224">
         <f>Paėmimas!L13</f>
         <v>0.05</v>
@@ -6741,7 +6746,7 @@
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="63"/>
       <c r="B14" s="64"/>
-      <c r="C14" s="279"/>
+      <c r="C14" s="259"/>
       <c r="D14" s="224">
         <f>Paėmimas!L14</f>
         <v>0.05</v>
@@ -6824,7 +6829,7 @@
         <f>Paėmimas!B19</f>
         <v>1</v>
       </c>
-      <c r="C19" s="277" t="str">
+      <c r="C19" s="257" t="str">
         <f>Paėmimas!C19</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -6876,7 +6881,7 @@
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="61"/>
       <c r="B20" s="23"/>
-      <c r="C20" s="278"/>
+      <c r="C20" s="258"/>
       <c r="D20" s="224">
         <f>Paėmimas!L20</f>
         <v>0.05</v>
@@ -6913,7 +6918,7 @@
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="61"/>
       <c r="B21" s="23"/>
-      <c r="C21" s="278"/>
+      <c r="C21" s="258"/>
       <c r="D21" s="224">
         <f>Paėmimas!L21</f>
         <v>0.05</v>
@@ -6950,7 +6955,7 @@
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="61"/>
       <c r="B22" s="23"/>
-      <c r="C22" s="278"/>
+      <c r="C22" s="258"/>
       <c r="D22" s="224">
         <f>Paėmimas!L22</f>
         <v>0.05</v>
@@ -6987,7 +6992,7 @@
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="61"/>
       <c r="B23" s="23"/>
-      <c r="C23" s="278"/>
+      <c r="C23" s="258"/>
       <c r="D23" s="224">
         <f>Paėmimas!L23</f>
         <v>0.05</v>
@@ -7024,7 +7029,7 @@
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24" s="61"/>
       <c r="B24" s="23"/>
-      <c r="C24" s="278"/>
+      <c r="C24" s="258"/>
       <c r="D24" s="224">
         <f>Paėmimas!L24</f>
         <v>0.05</v>
@@ -7061,7 +7066,7 @@
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25" s="61"/>
       <c r="B25" s="23"/>
-      <c r="C25" s="278"/>
+      <c r="C25" s="258"/>
       <c r="D25" s="224">
         <f>Paėmimas!L25</f>
         <v>0.05</v>
@@ -7098,7 +7103,7 @@
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26" s="61"/>
       <c r="B26" s="23"/>
-      <c r="C26" s="278"/>
+      <c r="C26" s="258"/>
       <c r="D26" s="224">
         <f>Paėmimas!L26</f>
         <v>0.05</v>
@@ -7135,7 +7140,7 @@
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27" s="63"/>
       <c r="B27" s="64"/>
-      <c r="C27" s="279"/>
+      <c r="C27" s="259"/>
       <c r="D27" s="224">
         <f>Paėmimas!L27</f>
         <v>0.05</v>
@@ -7293,7 +7298,7 @@
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.39370078740157483" right="0" top="0.74803149606299213" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="68" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="97" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddFooter>&amp;CPuslapių &amp;P &amp;R&amp;"Times New Roman,Paryškintasis"E5-5_02         
 2022-02-01, EV</oddFooter>
@@ -7330,10 +7335,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="281" t="s">
+      <c r="C1" s="261" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="281"/>
+      <c r="D1" s="261"/>
       <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -7586,12 +7591,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C1" s="281" t="s">
+      <c r="C1" s="261" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="281"/>
-      <c r="E1" s="281"/>
-      <c r="F1" s="281"/>
+      <c r="D1" s="261"/>
+      <c r="E1" s="261"/>
+      <c r="F1" s="261"/>
     </row>
     <row r="2" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="283" t="s">
@@ -7613,49 +7618,49 @@
       <c r="O2" s="283"/>
     </row>
     <row r="4" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="292" t="s">
+      <c r="A4" s="287" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="292" t="s">
+      <c r="B4" s="287" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="289" t="s">
+      <c r="C4" s="298" t="s">
         <v>84</v>
       </c>
-      <c r="D4" s="289" t="s">
+      <c r="D4" s="298" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="289" t="s">
+      <c r="E4" s="298" t="s">
         <v>86</v>
       </c>
-      <c r="F4" s="289"/>
-      <c r="G4" s="289"/>
-      <c r="H4" s="289" t="s">
+      <c r="F4" s="298"/>
+      <c r="G4" s="298"/>
+      <c r="H4" s="298" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="296" t="s">
+      <c r="I4" s="291" t="s">
         <v>87</v>
       </c>
-      <c r="J4" s="291" t="s">
+      <c r="J4" s="286" t="s">
         <v>88</v>
       </c>
-      <c r="K4" s="291"/>
-      <c r="L4" s="291"/>
-      <c r="M4" s="298" t="s">
+      <c r="K4" s="286"/>
+      <c r="L4" s="286"/>
+      <c r="M4" s="293" t="s">
         <v>89</v>
       </c>
-      <c r="N4" s="291" t="s">
+      <c r="N4" s="286" t="s">
         <v>15</v>
       </c>
-      <c r="O4" s="294" t="s">
+      <c r="O4" s="289" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="293"/>
-      <c r="B5" s="293"/>
-      <c r="C5" s="290"/>
-      <c r="D5" s="289"/>
+      <c r="A5" s="288"/>
+      <c r="B5" s="288"/>
+      <c r="C5" s="299"/>
+      <c r="D5" s="298"/>
       <c r="E5" s="120">
         <v>1</v>
       </c>
@@ -7665,8 +7670,8 @@
       <c r="G5" s="120">
         <v>3</v>
       </c>
-      <c r="H5" s="289"/>
-      <c r="I5" s="297"/>
+      <c r="H5" s="298"/>
+      <c r="I5" s="292"/>
       <c r="J5" s="12">
         <v>1</v>
       </c>
@@ -7676,16 +7681,16 @@
       <c r="L5" s="12">
         <v>3</v>
       </c>
-      <c r="M5" s="299"/>
-      <c r="N5" s="291"/>
-      <c r="O5" s="295"/>
+      <c r="M5" s="294"/>
+      <c r="N5" s="286"/>
+      <c r="O5" s="290"/>
     </row>
     <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="251">
         <f>Paėmimas!B6</f>
         <v>1</v>
       </c>
-      <c r="B6" s="286" t="str">
+      <c r="B6" s="295" t="str">
         <f>Paėmimas!C6</f>
         <v>UAB ,,Ekopartneris", L. Ivinskio g. 65, Kaunas. Katilinė. Taršos šaltinis  Nr. 001.</v>
       </c>
@@ -7735,7 +7740,7 @@
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="34"/>
-      <c r="B7" s="287"/>
+      <c r="B7" s="296"/>
       <c r="C7" s="33">
         <v>2</v>
       </c>
@@ -7772,7 +7777,7 @@
     </row>
     <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="34"/>
-      <c r="B8" s="287"/>
+      <c r="B8" s="296"/>
       <c r="C8" s="33"/>
       <c r="D8" s="92"/>
       <c r="E8" s="201"/>
@@ -7792,7 +7797,7 @@
     </row>
     <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A9" s="34"/>
-      <c r="B9" s="287"/>
+      <c r="B9" s="296"/>
       <c r="C9" s="33">
         <v>3</v>
       </c>
@@ -7829,7 +7834,7 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="34"/>
-      <c r="B10" s="287"/>
+      <c r="B10" s="296"/>
       <c r="C10" s="33"/>
       <c r="D10" s="92"/>
       <c r="E10" s="201"/>
@@ -7846,7 +7851,7 @@
     </row>
     <row r="11" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A11" s="34"/>
-      <c r="B11" s="287"/>
+      <c r="B11" s="296"/>
       <c r="C11" s="33">
         <v>41</v>
       </c>
@@ -7882,7 +7887,7 @@
     </row>
     <row r="12" spans="1:16" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="34"/>
-      <c r="B12" s="287"/>
+      <c r="B12" s="296"/>
       <c r="C12" s="115" t="s">
         <v>46</v>
       </c>
@@ -7918,7 +7923,7 @@
     </row>
     <row r="13" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A13" s="34"/>
-      <c r="B13" s="287"/>
+      <c r="B13" s="296"/>
       <c r="C13" s="116" t="s">
         <v>47</v>
       </c>
@@ -7954,7 +7959,7 @@
     </row>
     <row r="14" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A14" s="34"/>
-      <c r="B14" s="287"/>
+      <c r="B14" s="296"/>
       <c r="C14" s="116" t="s">
         <v>48</v>
       </c>
@@ -7990,7 +7995,7 @@
     </row>
     <row r="15" spans="1:16" ht="17" x14ac:dyDescent="0.45">
       <c r="A15" s="34"/>
-      <c r="B15" s="287"/>
+      <c r="B15" s="296"/>
       <c r="C15" s="117" t="s">
         <v>49</v>
       </c>
@@ -8026,7 +8031,7 @@
     </row>
     <row r="16" spans="1:16" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="22"/>
-      <c r="B16" s="288"/>
+      <c r="B16" s="297"/>
       <c r="C16" s="33"/>
       <c r="D16" s="95"/>
       <c r="E16" s="21"/>
@@ -8060,6 +8065,11 @@
     </sortState>
   </autoFilter>
   <mergeCells count="14">
+    <mergeCell ref="B6:B16"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="H4:H5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A2:O2"/>
@@ -8069,11 +8079,6 @@
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="M4:M5"/>
-    <mergeCell ref="B6:B16"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -8149,6 +8154,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokumentas" ma:contentTypeID="0x010100BAB57CF81AE55C4698AAD22D302297F0" ma:contentTypeVersion="18" ma:contentTypeDescription="Kurkite naują dokumentą." ma:contentTypeScope="" ma:versionID="49ab401eb4052690d2a2629974c22fd6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="453e7e53-5eb2-45cf-b2ab-34c867e554b8" xmlns:ns3="aa0d983d-359a-438c-9953-3af1a8ac0831" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ab9969d50e0b13c63bc5bd0499c928dc" ns2:_="" ns3:_="">
     <xsd:import namespace="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
@@ -8403,28 +8428,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="453e7e53-5eb2-45cf-b2ab-34c867e554b8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="aa0d983d-359a-438c-9953-3af1a8ac0831" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A76AEC4-30EA-47BC-874D-3E7B98533503}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8436,12 +8448,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A76AEC4-30EA-47BC-874D-3E7B98533503}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
     <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Suskaičiuota viskas iki izokinetiškumo parinkimo
</commit_message>
<xml_diff>
--- a/Ivestis2.xlsx
+++ b/Ivestis2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="Šios_darbaknygės" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agentura2020.sharepoint.com/sites/VidurioLietuvosaplinkostyrimuskyrius/Bendrai naudojami dokumentai/EB7-014 Darbuotojų failai/Tomo/Python 3.14.3/Skaiciavimai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="265" documentId="13_ncr:1_{D8ED3FA4-1188-4E70-924F-660A50F19C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95D2F3A6-D36A-4B1D-863B-1FF9AD1318ED}"/>
+  <xr:revisionPtr revIDLastSave="267" documentId="13_ncr:1_{D8ED3FA4-1188-4E70-924F-660A50F19C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C12CB74-2836-4FC7-B198-2453F28E0752}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="3" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="821" firstSheet="1" activeTab="4" xr2:uid="{B097D0E3-85A4-46F7-964F-ABE00A6941B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Compatibility Report" sheetId="4" state="hidden" r:id="rId1"/>
@@ -4396,7 +4396,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="YnNuFyjIZWP4o8siiNLOxJuXYMQvqdvZ9OrGGKpnMs1jyahS3pGpSVhE713S/7NZQvFDz0ZfCGMwTjhjC08CdQ==" saltValue="gCAgvRWICbIOkCsyhMCWFQ==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="11">
     <mergeCell ref="AB20:AB21"/>
     <mergeCell ref="D2:Z2"/>
@@ -6604,7 +6604,7 @@
       <c r="J30" s="96"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="Q7zQYUs0oFV/Gufx4DvoPWUpCjgOT2OzgA8jP4+OReQfg8sPFVBJlJin6okpsn/bA60CDJSSySZP7yIIZexC0Q==" saltValue="I0m09WVlXZjQAlrY7KWzKQ==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="4">
     <mergeCell ref="C2:M2"/>
     <mergeCell ref="C1:D1"/>
@@ -7696,15 +7696,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1A676EA-343E-4342-8BA5-7010E1EF44D6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1A676EA-343E-4342-8BA5-7010E1EF44D6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709F4DDD-DF1A-450D-8BF1-976CA47CFD58}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="453e7e53-5eb2-45cf-b2ab-34c867e554b8"/>
     <ds:schemaRef ds:uri="aa0d983d-359a-438c-9953-3af1a8ac0831"/>
   </ds:schemaRefs>
 </ds:datastoreItem>

</xml_diff>